<commit_message>
atualização das duplicatas e formatos
</commit_message>
<xml_diff>
--- a/Cronograma_VESPERTINO.xlsx
+++ b/Cronograma_VESPERTINO.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L19"/>
+  <dimension ref="A1:M19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -461,27 +461,32 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
+          <t>COORIENTADOR</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
           <t>ALUNO_ORIENTADO</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>TITULO TCC</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>MEMBRO 1</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>MEMBRO 2</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>MEMBRO 3</t>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>TILSP</t>
         </is>
       </c>
     </row>
@@ -519,27 +524,30 @@
           <t>Giuliano Lellis Ito Santos</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="H2" t="n">
+        <v/>
+      </c>
+      <c r="I2" t="inlineStr">
         <is>
           <t>Maria Jacinta Pfeiffer</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>O tempo como fator de conversão: Uma canção de natal de Charles Dickens</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>Eunice de Morais</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>Patricia Barreto Mainardi Maeso</t>
         </is>
       </c>
-      <c r="L2" t="n">
+      <c r="M2" t="n">
         <v/>
       </c>
     </row>
@@ -577,33 +585,36 @@
           <t>Letícia Fraga</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="H3" t="n">
+        <v/>
+      </c>
+      <c r="I3" t="inlineStr">
         <is>
           <t>Elise Thaynara-Yvian Mendes Christofoli</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>Variedade de francês no ensino de FLE no Brasil e Lei 10.639/03: uma discussão necessária</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>Djane Antonucci Correa</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>Ione da Silva Jovino</t>
         </is>
       </c>
-      <c r="L3" t="n">
+      <c r="M3" t="n">
         <v/>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>22</v>
+        <v>5</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -617,51 +628,54 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>13:50</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>B204</t>
+          <t>B202</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>LIBRAS</t>
+          <t>LITERATURA</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Rúbia Carla da Silva</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>Amanda Rafaelly de Paula Rocha</t>
-        </is>
+          <t>Giuliano Lellis Ito Santos</t>
+        </is>
+      </c>
+      <c r="H4" t="n">
+        <v/>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>COMUNICAÇÃO SOCIAL HÁPTICA: LÍNGUA, INTERAÇÃO E PRODUÇÃO DE SENTIDOS NO CONTEXTO DA SURDOCEGUEIRA</t>
+          <t>Rodrigo Paes</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Andressa França</t>
+          <t>A representação da morte em Pathologic 2 (2019)</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Pâmela Cristina Pereira Gonzaga</t>
-        </is>
-      </c>
-      <c r="L4" t="n">
+          <t>Daiane Cristina Pereira</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Jane Kelly de Oliveira</t>
+        </is>
+      </c>
+      <c r="M4" t="n">
         <v/>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -680,46 +694,53 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>B202</t>
+          <t>B203</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>LITERATURA</t>
+          <t>LIBRAS</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Giuliano Lellis Ito Santos</t>
+          <t xml:space="preserve">Rúbia Carla da Silva </t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Rodrigo Paes</t>
+          <t>Djane Antonucci Correa</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>A representação da morte em Pathologic 2 (2019)</t>
+          <t>Marcos Vinicius Matias</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Daiane Cristina Pereira</t>
+          <t>ENTRE MÃOS E TERRITÓRIOS: LÍNGUAS INDÍGENAS DE SINAIS E SINGULARIDADES/IDENTIDADES DE INDÍGENAS SURDOS</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Jane Kelly de Oliveira</t>
-        </is>
-      </c>
-      <c r="L5" t="n">
-        <v/>
+          <t>Shirley Vilhalva</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Letícia Fraga</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Marcelo Oliveira Bleme</t>
+        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>25</v>
+        <v>4</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -733,53 +754,54 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>16:10</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>B203</t>
+          <t>B202</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>LIBRAS</t>
+          <t>LITERATURA</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Rúbia Carla da Silva e Djane Antonucci Correa</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>Marcos Vinicius Matias</t>
-        </is>
+          <t>Giuliano Lellis Ito Santos</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v/>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>ENTRE MÃOS E TERRITÓRIOS: LÍNGUAS INDÍGENAS DE SINAIS E SINGULARIDADES/IDENTIDADES DE INDÍGENAS SURDOS</t>
+          <t>Isabela Delgobo Champoski</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Shirley Vilhalva</t>
+          <t>A proibição do celular em sala de aula: análise da aplicação da Lei 15.100/2025 em escolas públicas (2024-2025)</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Letícia Fraga</t>
+          <t>Ályda Henrietta Zomer</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>TILSP - Marcelo Oliveira Bleme</t>
-        </is>
+          <t>Silvely Brandes</t>
+        </is>
+      </c>
+      <c r="M6" t="n">
+        <v/>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>37</v>
+        <v>1</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -793,53 +815,54 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>16:10</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>B204</t>
+          <t>B203</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>LIBRAS</t>
+          <t>LINGUÍSTICA</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Andressa França</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>CLAUDINEIA MACHADO DE OLIVEIRA</t>
-        </is>
+          <t>Letícia Fraga</t>
+        </is>
+      </c>
+      <c r="H7" t="n">
+        <v/>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Aquisição tardia da Libras, escolarização e identidade surda: análise da narrativa de uma professora surda do Paraná</t>
+          <t>Henrique Leal Rodrigues</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Katherine Fischer</t>
+          <t>LUZ POR ENTRE AS NUVENS: A LITERATURA INFANTOJUVENIL COMO MEDIADORA DE TEMAS CONSIDERADOS SENSÍVEIS NA ESCOLA</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Marcelo Elisio Vasicki</t>
+          <t>Djane Antonucci Correa</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>Cristiane Rocha</t>
-        </is>
+          <t>Ligia Paula Couto</t>
+        </is>
+      </c>
+      <c r="M7" t="n">
+        <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>4</v>
+        <v>59</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -858,50 +881,53 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>B202</t>
+          <t>B204</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>LITERATURA</t>
+          <t>LINGUÍSTICA</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Giuliano Lellis Ito Santos</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>Isabela Delgobo Champoski</t>
-        </is>
+          <t>Rosita Maria Bastos dos Santos</t>
+        </is>
+      </c>
+      <c r="H8" t="n">
+        <v/>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>A proibição do celular em sala de aula: análise da aplicação da Lei 15.100/2025 em escolas públicas (2024-2025)</t>
+          <t>João Pedro Mendes Santos</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Ályda Henrietta Zomer</t>
+          <t>Entre a universidade e a sala de aula: memórias e reflexões sobre a construção docente</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Silvely Brandes</t>
-        </is>
-      </c>
-      <c r="L8" t="n">
+          <t>Audrey Pietrobeli de Souza</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Eliane Santos Raupp</t>
+        </is>
+      </c>
+      <c r="M8" t="n">
         <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>1</v>
+        <v>28</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Segunda</t>
+          <t>Terça</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -911,12 +937,12 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>16:10</t>
+          <t>13:50</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>B203</t>
+          <t>B201</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -926,30 +952,33 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Letícia Fraga</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>Henrique Leal Rodrigues</t>
-        </is>
+          <t>Silvely Brandes</t>
+        </is>
+      </c>
+      <c r="H9" t="n">
+        <v/>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>LUZ POR ENTRE AS NUVENS: A LITERATURA INFANTOJUVENIL COMO MEDIADORA DE TEMAS CONSIDERADOS SENSÍVEIS NA ESCOLA</t>
+          <t>Debora Santos Resende</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Djane Antonucci Correa</t>
+          <t>AS PLATAFORMAS DE ENSINO DE INGLÊS DA REDE PÚBLICA PARANAENSE FRENTE AOS DOCUMENTOS OFICIAIS</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Ligia Paula Couto</t>
-        </is>
-      </c>
-      <c r="L9" t="n">
+          <t>Isabel Cristina Vollet Marson</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Ronna Freitas</t>
+        </is>
+      </c>
+      <c r="M9" t="n">
         <v/>
       </c>
     </row>
@@ -959,7 +988,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Segunda</t>
+          <t>Terça</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -969,12 +998,12 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>16:10</t>
+          <t>13:50</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>B204</t>
+          <t>B202</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -987,35 +1016,38 @@
           <t>Rúbia Carla da Silva</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="H10" t="n">
+        <v/>
+      </c>
+      <c r="I10" t="inlineStr">
         <is>
           <t>Thyelle Francine Braz de Proença</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="J10" t="inlineStr">
         <is>
           <t>A IMPORTÂNCIA DA LITERATURA SURDA PARA O ENSINO DE LIBRAS</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="K10" t="inlineStr">
         <is>
           <t>Mariana de Oliveira Ferreira</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr">
+      <c r="L10" t="inlineStr">
         <is>
           <t>Vinícius Heitor Pereira</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>TILSP - Cristiane Ribeiro Rocha</t>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Cristiane Ribeiro Rocha</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -1034,7 +1066,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>B202</t>
+          <t>B203</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1044,36 +1076,39 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Silvely Brandes</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>Debora Santos Resende</t>
-        </is>
+          <t>Dilma Heloisa Santos</t>
+        </is>
+      </c>
+      <c r="H11" t="n">
+        <v/>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>AS PLATAFORMAS DE ENSINO DE INGLÊS DA REDE PÚBLICA PARANAENSE FRENTE AOS DOCUMENTOS OFICIAIS</t>
+          <t>Naiara Karin de Ramos</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Isabel Cristina Vollet Marson</t>
+          <t>PRIVILÉGIO E NEGAÇÃO: MANIFESTAÇÕES DA BRANQUITUDE NA PÓS-GRADUAÇÃO DA UNIVERSIDADE ESTADUAL DE PONTA GROSSA</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Ronna Freitas</t>
-        </is>
-      </c>
-      <c r="L11" t="n">
+          <t>Lucimar Araujo Braga</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>Gisele de Fátima do Prado</t>
+        </is>
+      </c>
+      <c r="M11" t="n">
         <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1092,46 +1127,49 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>B203</t>
+          <t>B204</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>LINGUÍSTICA</t>
+          <t>LITERATURA</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Dilma Heloisa Santos</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>Naiara Karin de Ramos</t>
-        </is>
+          <t>Keli Cristina Pacheco</t>
+        </is>
+      </c>
+      <c r="H12" t="n">
+        <v/>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>PRIVILÉGIO E NEGAÇÃO: MANIFESTAÇÕES DA BRANQUITUDE NA PÓS-GRADUAÇÃO DA UNIVERSIDADE ESTADUAL DE PONTA GROSSA</t>
+          <t>Gustavo Henrique do Nascimento</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Lucimar Araujo Braga</t>
+          <t>Entre Máscaras e Desejos: A Construção da Personagem Transgênero em Stella Manhattan, de Silviano Santiago</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Gisele de Fátima do Prado</t>
-        </is>
-      </c>
-      <c r="L12" t="n">
+          <t>Joana dArc Martins Pupo</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Giuliano Lellis Ito Santos </t>
+        </is>
+      </c>
+      <c r="M12" t="n">
         <v/>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -1145,51 +1183,54 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>13:50</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>B204</t>
+          <t>B201</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>LITERATURA</t>
+          <t>LINGUÍSTICA</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Keli Cristina Pacheco</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>Gustavo Henrique do Nascimento</t>
-        </is>
+          <t>Silvely Brandes</t>
+        </is>
+      </c>
+      <c r="H13" t="n">
+        <v/>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Entre Máscaras e Desejos: A Construção da Personagem Transgênero em Stella Manhattan, de Silviano Santiago</t>
+          <t>PEDRO MEYER KOPP</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Joana dArc Martins Pupo</t>
+          <t>A TRADUÇÃO AUTOMÁTICA DENTRO DE JOGOS ELETRÔNICOS NA PLATAFORMA ROBLOX: UMA ANÁLISE QUALITATIVA</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Giuliano Lellis Ito Santos </t>
-        </is>
-      </c>
-      <c r="L13" t="n">
+          <t xml:space="preserve">Álvaro Kasuaki Fujihara </t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Marcos Barbosa Carreira </t>
+        </is>
+      </c>
+      <c r="M13" t="n">
         <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>58</v>
+        <v>22</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -1213,35 +1254,38 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>LINGUÍSTICA</t>
+          <t>LIBRAS</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Rosita Maria Bastos dos Santos</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>Martha Caixeta Cardoso</t>
-        </is>
+          <t>Rúbia Carla da Silva</t>
+        </is>
+      </c>
+      <c r="H14" t="n">
+        <v/>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>A ESCRITA AUTORAL COMO ESTRATÉGIA PEDAGÓGICA NA LEITURA E PRODUÇÃO DE TEXTOS: UM RELATO DE EXPERIÊNCIA NO PROJETO DE EXTENSÃO</t>
+          <t>Amanda Rafaelly de Paula Rocha</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Eliane Santos Raupp</t>
+          <t>COMUNICAÇÃO SOCIAL HÁPTICA: LÍNGUA, INTERAÇÃO E PRODUÇÃO DE SENTIDOS NO CONTEXTO DA SURDOCEGUEIRA</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Djane Antonucci Correa</t>
-        </is>
-      </c>
-      <c r="L14" t="n">
+          <t>Andressa França</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>Pâmela Cristina Pereira Gonzaga</t>
+        </is>
+      </c>
+      <c r="M14" t="n">
         <v/>
       </c>
     </row>
@@ -1279,27 +1323,30 @@
           <t>Ligia Paula Couto</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
+      <c r="H15" t="n">
+        <v/>
+      </c>
+      <c r="I15" t="inlineStr">
         <is>
           <t>GRACIELY CRISTINY MATOS VIEIRA</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr">
+      <c r="J15" t="inlineStr">
         <is>
           <t xml:space="preserve">O ESTUDO DO CONCEITO “QUILOMBOLA” COMO CHAVE PARA COMPREENDER A IDENTIDADE E EDUCAÇÃO ESCOLAR QUILOMBOLA </t>
         </is>
       </c>
-      <c r="J15" t="inlineStr">
+      <c r="K15" t="inlineStr">
         <is>
           <t>Ione da Silva Jovino</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr">
+      <c r="L15" t="inlineStr">
         <is>
           <t>Benedito Florindo de Freitas Júnior</t>
         </is>
       </c>
-      <c r="L15" t="n">
+      <c r="M15" t="n">
         <v/>
       </c>
     </row>
@@ -1337,33 +1384,36 @@
           <t>Jane Kelly de Oliveira</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
+      <c r="H16" t="n">
+        <v/>
+      </c>
+      <c r="I16" t="inlineStr">
         <is>
           <t>Letícia Fukae da Silva</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr">
+      <c r="J16" t="inlineStr">
         <is>
           <t xml:space="preserve">Sombras do que fui: a cidade e o feminino frente à guerra em As Troianas, de Eurípides </t>
         </is>
       </c>
-      <c r="J16" t="inlineStr">
+      <c r="K16" t="inlineStr">
         <is>
           <t>Keli Cristina Pacheco</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr">
+      <c r="L16" t="inlineStr">
         <is>
           <t>Daiane Cristina Pereira</t>
         </is>
       </c>
-      <c r="L16" t="n">
+      <c r="M16" t="n">
         <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>59</v>
+        <v>37</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1387,41 +1437,46 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>LINGUÍSTICA</t>
+          <t>LIBRAS</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Rosita Maria Bastos dos Santos</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>João Pedro Mendes Santos</t>
-        </is>
+          <t>Andressa França</t>
+        </is>
+      </c>
+      <c r="H17" t="n">
+        <v/>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Entre a universidade e a sala de aula: memórias e reflexões sobre a construção docente</t>
+          <t>CLAUDINEIA MACHADO DE OLIVEIRA</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>Audrey Pietrobeli de Souza</t>
+          <t>Aquisição tardia da Libras, escolarização e identidade surda: análise da narrativa de uma professora surda do Paraná</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>Eliane Santos Raupp</t>
-        </is>
-      </c>
-      <c r="L17" t="n">
-        <v/>
+          <t>Katherine Fischer</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>Marcelo Elisio Vasicki</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>Cristiane Ribeiro Rocha</t>
+        </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>27</v>
+        <v>58</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1450,30 +1505,33 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Silvely Brandes</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>PEDRO MEYER KOPP</t>
-        </is>
+          <t>Rosita Maria Bastos dos Santos</t>
+        </is>
+      </c>
+      <c r="H18" t="n">
+        <v/>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>A TRADUÇÃO AUTOMÁTICA DENTRO DE JOGOS ELETRÔNICOS NA PLATAFORMA ROBLOX: UMA ANÁLISE QUALITATIVA</t>
+          <t>Martha Caixeta Cardoso</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Alvaro Kasuaki Fujihara </t>
+          <t>A ESCRITA AUTORAL COMO ESTRATÉGIA PEDAGÓGICA NA LEITURA E PRODUÇÃO DE TEXTOS: UM RELATO DE EXPERIÊNCIA NO PROJETO DE EXTENSÃO</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Marcos Barbosa Carreira </t>
-        </is>
-      </c>
-      <c r="L18" t="n">
+          <t>Eliane Santos Raupp</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>Djane Antonucci Correa</t>
+        </is>
+      </c>
+      <c r="M18" t="n">
         <v/>
       </c>
     </row>
@@ -1511,27 +1569,30 @@
           <t>Joana dArc Martins Pupo</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr">
+      <c r="H19" t="n">
+        <v/>
+      </c>
+      <c r="I19" t="inlineStr">
         <is>
           <t>Ananda Carolina Ribeiro</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr">
+      <c r="J19" t="inlineStr">
         <is>
           <t>A Filosofia Educacional de Mary Wollstonecraft em Original Stories from real life (1788) e em A Vindication of the Rights of Woman (1792)</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>Clóris Porto Torquato</t>
-        </is>
-      </c>
       <c r="K19" t="inlineStr">
         <is>
+          <t>Cloris Porto Torquato</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
           <t>Daiane Cristina Pereira</t>
         </is>
       </c>
-      <c r="L19" t="n">
+      <c r="M19" t="n">
         <v/>
       </c>
     </row>
@@ -1546,7 +1607,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H58"/>
+  <dimension ref="A1:H59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1594,7 +1655,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Alvaro Kasuaki Fujihara</t>
+          <t>Andressa França</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1609,12 +1670,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>16:10</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>B203</t>
+          <t>B202</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -1624,12 +1685,12 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>PEDRO MEYER KOPP</t>
+          <t>Amanda Rafaelly de Paula Rocha</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>A TRADUÇÃO AUTOMÁTICA DENTRO DE JOGOS ELETRÔNICOS NA PLATAFORMA ROBLOX: UMA ANÁLISE QUALITATIVA</t>
+          <t>COMUNICAÇÃO SOCIAL HÁPTICA: LÍNGUA, INTERAÇÃO E PRODUÇÃO DE SENTIDOS NO CONTEXTO DA SURDOCEGUEIRA</t>
         </is>
       </c>
     </row>
@@ -1641,7 +1702,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Segunda</t>
+          <t>Terça</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1651,34 +1712,34 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>13:50</t>
+          <t>16:10</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>B204</t>
+          <t>B202</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Membro</t>
+          <t>Orientador</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Amanda Rafaelly de Paula Rocha</t>
+          <t>CLAUDINEIA MACHADO DE OLIVEIRA</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>COMUNICAÇÃO SOCIAL HÁPTICA: LÍNGUA, INTERAÇÃO E PRODUÇÃO DE SENTIDOS NO CONTEXTO DA SURDOCEGUEIRA</t>
+          <t>Aquisição tardia da Libras, escolarização e identidade surda: análise da narrativa de uma professora surda do Paraná</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Andressa França</t>
+          <t>Audrey Pietrobeli de Souza</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1693,7 +1754,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>16:10</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -1703,24 +1764,24 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Orientador</t>
+          <t>Membro</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>CLAUDINEIA MACHADO DE OLIVEIRA</t>
+          <t>João Pedro Mendes Santos</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Aquisição tardia da Libras, escolarização e identidade surda: análise da narrativa de uma professora surda do Paraná</t>
+          <t>Entre a universidade e a sala de aula: memórias e reflexões sobre a construção docente</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Audrey Pietrobeli de Souza</t>
+          <t>Benedito Florindo de Freitas Júnior</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1735,12 +1796,12 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>16:10</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>B202</t>
+          <t>B203</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -1750,19 +1811,19 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>João Pedro Mendes Santos</t>
+          <t>GRACIELY CRISTINY MATOS VIEIRA</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Entre a universidade e a sala de aula: memórias e reflexões sobre a construção docente</t>
+          <t xml:space="preserve">O ESTUDO DO CONCEITO “QUILOMBOLA” COMO CHAVE PARA COMPREENDER A IDENTIDADE E EDUCAÇÃO ESCOLAR QUILOMBOLA </t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Benedito Florindo de Freitas Júnior</t>
+          <t>Cloris Porto Torquato</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1777,12 +1838,12 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>16:10</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>B203</t>
+          <t>B204</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -1792,19 +1853,19 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>GRACIELY CRISTINY MATOS VIEIRA</t>
+          <t>Ananda Carolina Ribeiro</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t xml:space="preserve">O ESTUDO DO CONCEITO “QUILOMBOLA” COMO CHAVE PARA COMPREENDER A IDENTIDADE E EDUCAÇÃO ESCOLAR QUILOMBOLA </t>
+          <t>A Filosofia Educacional de Mary Wollstonecraft em Original Stories from real life (1788) e em A Vindication of the Rights of Woman (1792)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Clóris Porto Torquato</t>
+          <t>Cristiane Ribeiro Rocha</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1819,39 +1880,39 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>16:10</t>
+          <t>13:50</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>B204</t>
+          <t>B202</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Membro</t>
+          <t>TILSP</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Ananda Carolina Ribeiro</t>
+          <t>Thyelle Francine Braz de Proença</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>A Filosofia Educacional de Mary Wollstonecraft em Original Stories from real life (1788) e em A Vindication of the Rights of Woman (1792)</t>
+          <t>A IMPORTÂNCIA DA LITERATURA SURDA PARA O ENSINO DE LIBRAS</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Cristiane Rocha</t>
+          <t>Cristiane Ribeiro Rocha</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Segunda</t>
+          <t>Terça</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1861,17 +1922,17 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>16:10</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>B204</t>
+          <t>B202</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Membro</t>
+          <t>TILSP</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -2113,7 +2174,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>16:10</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -2123,17 +2184,17 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Membro</t>
+          <t>Coorientador</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Henrique Leal Rodrigues</t>
+          <t>Marcos Vinicius Matias</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>LUZ POR ENTRE AS NUVENS: A LITERATURA INFANTOJUVENIL COMO MEDIADORA DE TEMAS CONSIDERADOS SENSÍVEIS NA ESCOLA</t>
+          <t>ENTRE MÃOS E TERRITÓRIOS: LÍNGUAS INDÍGENAS DE SINAIS E SINGULARIDADES/IDENTIDADES DE INDÍGENAS SURDOS</t>
         </is>
       </c>
     </row>
@@ -2145,7 +2206,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Terça</t>
+          <t>Segunda</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -2155,12 +2216,12 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>16:10</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>B202</t>
+          <t>B203</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -2170,19 +2231,19 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Martha Caixeta Cardoso</t>
+          <t>Henrique Leal Rodrigues</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>A ESCRITA AUTORAL COMO ESTRATÉGIA PEDAGÓGICA NA LEITURA E PRODUÇÃO DE TEXTOS: UM RELATO DE EXPERIÊNCIA NO PROJETO DE EXTENSÃO</t>
+          <t>LUZ POR ENTRE AS NUVENS: A LITERATURA INFANTOJUVENIL COMO MEDIADORA DE TEMAS CONSIDERADOS SENSÍVEIS NA ESCOLA</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Eliane Santos Raupp</t>
+          <t>Djane Antonucci Correa</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2197,12 +2258,12 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>16:10</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>B202</t>
+          <t>B203</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -2229,7 +2290,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Terça</t>
+          <t>Segunda</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -2244,7 +2305,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>B202</t>
+          <t>B204</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -2266,12 +2327,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Eunice de Morais</t>
+          <t>Eliane Santos Raupp</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Segunda</t>
+          <t>Terça</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -2281,12 +2342,12 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>13:50</t>
+          <t>16:10</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>B202</t>
+          <t>B203</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -2296,24 +2357,24 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Maria Jacinta Pfeiffer</t>
+          <t>Martha Caixeta Cardoso</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>O tempo como fator de conversão: Uma canção de natal de Charles Dickens</t>
+          <t>A ESCRITA AUTORAL COMO ESTRATÉGIA PEDAGÓGICA NA LEITURA E PRODUÇÃO DE TEXTOS: UM RELATO DE EXPERIÊNCIA NO PROJETO DE EXTENSÃO</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Gisele de Fátima do Prado</t>
+          <t>Eunice de Morais</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Terça</t>
+          <t>Segunda</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -2328,7 +2389,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>B203</t>
+          <t>B202</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -2338,24 +2399,24 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Naiara Karin de Ramos</t>
+          <t>Maria Jacinta Pfeiffer</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>PRIVILÉGIO E NEGAÇÃO: MANIFESTAÇÕES DA BRANQUITUDE NA PÓS-GRADUAÇÃO DA UNIVERSIDADE ESTADUAL DE PONTA GROSSA</t>
+          <t>O tempo como fator de conversão: Uma canção de natal de Charles Dickens</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Giuliano Lellis Ito Santos</t>
+          <t>Gisele de Fátima do Prado</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Segunda</t>
+          <t>Terça</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -2370,22 +2431,22 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>B202</t>
+          <t>B203</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Orientador</t>
+          <t>Membro</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Maria Jacinta Pfeiffer</t>
+          <t>Naiara Karin de Ramos</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>O tempo como fator de conversão: Uma canção de natal de Charles Dickens</t>
+          <t>PRIVILÉGIO E NEGAÇÃO: MANIFESTAÇÕES DA BRANQUITUDE NA PÓS-GRADUAÇÃO DA UNIVERSIDADE ESTADUAL DE PONTA GROSSA</t>
         </is>
       </c>
     </row>
@@ -2407,7 +2468,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>13:50</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -2422,12 +2483,12 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Rodrigo Paes</t>
+          <t>Maria Jacinta Pfeiffer</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>A representação da morte em Pathologic 2 (2019)</t>
+          <t>O tempo como fator de conversão: Uma canção de natal de Charles Dickens</t>
         </is>
       </c>
     </row>
@@ -2449,7 +2510,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>16:10</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -2464,12 +2525,12 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Isabela Delgobo Champoski</t>
+          <t>Rodrigo Paes</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>A proibição do celular em sala de aula: análise da aplicação da Lei 15.100/2025 em escolas públicas (2024-2025)</t>
+          <t>A representação da morte em Pathologic 2 (2019)</t>
         </is>
       </c>
     </row>
@@ -2481,7 +2542,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Terça</t>
+          <t>Segunda</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -2491,39 +2552,39 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>13:50</t>
+          <t>16:10</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>B204</t>
+          <t>B202</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Membro</t>
+          <t>Orientador</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Gustavo Henrique do Nascimento</t>
+          <t>Isabela Delgobo Champoski</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>Entre Máscaras e Desejos: A Construção da Personagem Transgênero em Stella Manhattan, de Silviano Santiago</t>
+          <t>A proibição do celular em sala de aula: análise da aplicação da Lei 15.100/2025 em escolas públicas (2024-2025)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Ione da Silva Jovino</t>
+          <t>Giuliano Lellis Ito Santos</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Segunda</t>
+          <t>Terça</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -2538,7 +2599,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>B203</t>
+          <t>B204</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -2548,12 +2609,12 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Elise Thaynara-Yvian Mendes Christofoli</t>
+          <t>Gustavo Henrique do Nascimento</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Variedade de francês no ensino de FLE no Brasil e Lei 10.639/03: uma discussão necessária</t>
+          <t>Entre Máscaras e Desejos: A Construção da Personagem Transgênero em Stella Manhattan, de Silviano Santiago</t>
         </is>
       </c>
     </row>
@@ -2565,7 +2626,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Terça</t>
+          <t>Segunda</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -2575,7 +2636,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>13:50</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -2590,19 +2651,19 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>GRACIELY CRISTINY MATOS VIEIRA</t>
+          <t>Elise Thaynara-Yvian Mendes Christofoli</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t xml:space="preserve">O ESTUDO DO CONCEITO “QUILOMBOLA” COMO CHAVE PARA COMPREENDER A IDENTIDADE E EDUCAÇÃO ESCOLAR QUILOMBOLA </t>
+          <t>Variedade de francês no ensino de FLE no Brasil e Lei 10.639/03: uma discussão necessária</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Isabel Cristina Vollet Marson</t>
+          <t>Ione da Silva Jovino</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -2617,12 +2678,12 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>13:50</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>B202</t>
+          <t>B203</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -2632,24 +2693,24 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Debora Santos Resende</t>
+          <t>GRACIELY CRISTINY MATOS VIEIRA</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>AS PLATAFORMAS DE ENSINO DE INGLÊS DA REDE PÚBLICA PARANAENSE FRENTE AOS DOCUMENTOS OFICIAIS</t>
+          <t xml:space="preserve">O ESTUDO DO CONCEITO “QUILOMBOLA” COMO CHAVE PARA COMPREENDER A IDENTIDADE E EDUCAÇÃO ESCOLAR QUILOMBOLA </t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Jane Kelly de Oliveira</t>
+          <t>Isabel Cristina Vollet Marson</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Segunda</t>
+          <t>Terça</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -2659,12 +2720,12 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>13:50</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>B202</t>
+          <t>B201</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -2674,12 +2735,12 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Rodrigo Paes</t>
+          <t>Debora Santos Resende</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>A representação da morte em Pathologic 2 (2019)</t>
+          <t>AS PLATAFORMAS DE ENSINO DE INGLÊS DA REDE PÚBLICA PARANAENSE FRENTE AOS DOCUMENTOS OFICIAIS</t>
         </is>
       </c>
     </row>
@@ -2691,7 +2752,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Terça</t>
+          <t>Segunda</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -2706,29 +2767,29 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>B204</t>
+          <t>B202</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Orientador</t>
+          <t>Membro</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Letícia Fukae da Silva</t>
+          <t>Rodrigo Paes</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sombras do que fui: a cidade e o feminino frente à guerra em As Troianas, de Eurípides </t>
+          <t>A representação da morte em Pathologic 2 (2019)</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Joana dArc Martins Pupo</t>
+          <t>Jane Kelly de Oliveira</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -2743,7 +2804,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>13:50</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -2753,17 +2814,17 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Membro</t>
+          <t>Orientador</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Gustavo Henrique do Nascimento</t>
+          <t>Letícia Fukae da Silva</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Entre Máscaras e Desejos: A Construção da Personagem Transgênero em Stella Manhattan, de Silviano Santiago</t>
+          <t xml:space="preserve">Sombras do que fui: a cidade e o feminino frente à guerra em As Troianas, de Eurípides </t>
         </is>
       </c>
     </row>
@@ -2785,7 +2846,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>16:10</t>
+          <t>13:50</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -2795,29 +2856,29 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Orientador</t>
+          <t>Membro</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Ananda Carolina Ribeiro</t>
+          <t>Gustavo Henrique do Nascimento</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>A Filosofia Educacional de Mary Wollstonecraft em Original Stories from real life (1788) e em A Vindication of the Rights of Woman (1792)</t>
+          <t>Entre Máscaras e Desejos: A Construção da Personagem Transgênero em Stella Manhattan, de Silviano Santiago</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Katherine Fischer</t>
+          <t>Joana dArc Martins Pupo</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Segunda</t>
+          <t>Terça</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -2827,7 +2888,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>16:10</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -2837,24 +2898,24 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Membro</t>
+          <t>Orientador</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>CLAUDINEIA MACHADO DE OLIVEIRA</t>
+          <t>Ananda Carolina Ribeiro</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Aquisição tardia da Libras, escolarização e identidade surda: análise da narrativa de uma professora surda do Paraná</t>
+          <t>A Filosofia Educacional de Mary Wollstonecraft em Original Stories from real life (1788) e em A Vindication of the Rights of Woman (1792)</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Keli Cristina Pacheco</t>
+          <t>Katherine Fischer</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2869,27 +2930,27 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>13:50</t>
+          <t>16:10</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>B204</t>
+          <t>B202</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Orientador</t>
+          <t>Membro</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Gustavo Henrique do Nascimento</t>
+          <t>CLAUDINEIA MACHADO DE OLIVEIRA</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Entre Máscaras e Desejos: A Construção da Personagem Transgênero em Stella Manhattan, de Silviano Santiago</t>
+          <t>Aquisição tardia da Libras, escolarização e identidade surda: análise da narrativa de uma professora surda do Paraná</t>
         </is>
       </c>
     </row>
@@ -2911,7 +2972,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>13:50</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -2921,29 +2982,29 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Membro</t>
+          <t>Orientador</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Letícia Fukae da Silva</t>
+          <t>Gustavo Henrique do Nascimento</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sombras do que fui: a cidade e o feminino frente à guerra em As Troianas, de Eurípides </t>
+          <t>Entre Máscaras e Desejos: A Construção da Personagem Transgênero em Stella Manhattan, de Silviano Santiago</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Letícia Fraga</t>
+          <t>Keli Cristina Pacheco</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Segunda</t>
+          <t>Terça</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -2953,27 +3014,27 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>13:50</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>B203</t>
+          <t>B204</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Orientador</t>
+          <t>Membro</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Elise Thaynara-Yvian Mendes Christofoli</t>
+          <t>Letícia Fukae da Silva</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Variedade de francês no ensino de FLE no Brasil e Lei 10.639/03: uma discussão necessária</t>
+          <t xml:space="preserve">Sombras do que fui: a cidade e o feminino frente à guerra em As Troianas, de Eurípides </t>
         </is>
       </c>
     </row>
@@ -2995,7 +3056,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>13:50</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -3005,17 +3066,17 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Membro</t>
+          <t>Orientador</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Marcos Vinicius Matias</t>
+          <t>Elise Thaynara-Yvian Mendes Christofoli</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>ENTRE MÃOS E TERRITÓRIOS: LÍNGUAS INDÍGENAS DE SINAIS E SINGULARIDADES/IDENTIDADES DE INDÍGENAS SURDOS</t>
+          <t>Variedade de francês no ensino de FLE no Brasil e Lei 10.639/03: uma discussão necessária</t>
         </is>
       </c>
     </row>
@@ -3037,7 +3098,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>16:10</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -3047,24 +3108,24 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Orientador</t>
+          <t>Membro</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Henrique Leal Rodrigues</t>
+          <t>Marcos Vinicius Matias</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>LUZ POR ENTRE AS NUVENS: A LITERATURA INFANTOJUVENIL COMO MEDIADORA DE TEMAS CONSIDERADOS SENSÍVEIS NA ESCOLA</t>
+          <t>ENTRE MÃOS E TERRITÓRIOS: LÍNGUAS INDÍGENAS DE SINAIS E SINGULARIDADES/IDENTIDADES DE INDÍGENAS SURDOS</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Ligia Paula Couto</t>
+          <t>Letícia Fraga</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -3089,7 +3150,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Membro</t>
+          <t>Orientador</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -3111,7 +3172,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Terça</t>
+          <t>Segunda</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -3121,7 +3182,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>16:10</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -3131,24 +3192,24 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Orientador</t>
+          <t>Membro</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>GRACIELY CRISTINY MATOS VIEIRA</t>
+          <t>Henrique Leal Rodrigues</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t xml:space="preserve">O ESTUDO DO CONCEITO “QUILOMBOLA” COMO CHAVE PARA COMPREENDER A IDENTIDADE E EDUCAÇÃO ESCOLAR QUILOMBOLA </t>
+          <t>LUZ POR ENTRE AS NUVENS: A LITERATURA INFANTOJUVENIL COMO MEDIADORA DE TEMAS CONSIDERADOS SENSÍVEIS NA ESCOLA</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Lucimar Araujo Braga</t>
+          <t>Ligia Paula Couto</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -3163,7 +3224,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>13:50</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -3173,29 +3234,29 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Membro</t>
+          <t>Orientador</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Naiara Karin de Ramos</t>
+          <t>GRACIELY CRISTINY MATOS VIEIRA</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>PRIVILÉGIO E NEGAÇÃO: MANIFESTAÇÕES DA BRANQUITUDE NA PÓS-GRADUAÇÃO DA UNIVERSIDADE ESTADUAL DE PONTA GROSSA</t>
+          <t xml:space="preserve">O ESTUDO DO CONCEITO “QUILOMBOLA” COMO CHAVE PARA COMPREENDER A IDENTIDADE E EDUCAÇÃO ESCOLAR QUILOMBOLA </t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Marcelo Elisio Vasicki</t>
+          <t>Lucimar Araujo Braga</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Segunda</t>
+          <t>Terça</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -3205,12 +3266,12 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>13:50</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>B204</t>
+          <t>B203</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -3220,19 +3281,19 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>CLAUDINEIA MACHADO DE OLIVEIRA</t>
+          <t>Naiara Karin de Ramos</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>Aquisição tardia da Libras, escolarização e identidade surda: análise da narrativa de uma professora surda do Paraná</t>
+          <t>PRIVILÉGIO E NEGAÇÃO: MANIFESTAÇÕES DA BRANQUITUDE NA PÓS-GRADUAÇÃO DA UNIVERSIDADE ESTADUAL DE PONTA GROSSA</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Marcos Barbosa Carreira</t>
+          <t>Marcelo Elisio Vasicki</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -3252,7 +3313,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>B203</t>
+          <t>B202</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -3262,19 +3323,19 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>PEDRO MEYER KOPP</t>
+          <t>CLAUDINEIA MACHADO DE OLIVEIRA</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>A TRADUÇÃO AUTOMÁTICA DENTRO DE JOGOS ELETRÔNICOS NA PLATAFORMA ROBLOX: UMA ANÁLISE QUALITATIVA</t>
+          <t>Aquisição tardia da Libras, escolarização e identidade surda: análise da narrativa de uma professora surda do Paraná</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Mariana de Oliveira Ferreira</t>
+          <t>Marcelo Oliveira Bleme</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -3289,39 +3350,39 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>16:10</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>B204</t>
+          <t>B203</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Membro</t>
+          <t>TILSP</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Thyelle Francine Braz de Proença</t>
+          <t>Marcos Vinicius Matias</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>A IMPORTÂNCIA DA LITERATURA SURDA PARA O ENSINO DE LIBRAS</t>
+          <t>ENTRE MÃOS E TERRITÓRIOS: LÍNGUAS INDÍGENAS DE SINAIS E SINGULARIDADES/IDENTIDADES DE INDÍGENAS SURDOS</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Patricia Barreto Mainardi Maeso</t>
+          <t>Marcos Barbosa Carreira</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Segunda</t>
+          <t>Terça</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -3331,12 +3392,12 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>13:50</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>B202</t>
+          <t>B201</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -3346,24 +3407,24 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Maria Jacinta Pfeiffer</t>
+          <t>PEDRO MEYER KOPP</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>O tempo como fator de conversão: Uma canção de natal de Charles Dickens</t>
+          <t>A TRADUÇÃO AUTOMÁTICA DENTRO DE JOGOS ELETRÔNICOS NA PLATAFORMA ROBLOX: UMA ANÁLISE QUALITATIVA</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Pâmela Cristina Pereira Gonzaga</t>
+          <t>Mariana de Oliveira Ferreira</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Segunda</t>
+          <t>Terça</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -3378,7 +3439,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>B204</t>
+          <t>B202</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -3388,24 +3449,24 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Amanda Rafaelly de Paula Rocha</t>
+          <t>Thyelle Francine Braz de Proença</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>COMUNICAÇÃO SOCIAL HÁPTICA: LÍNGUA, INTERAÇÃO E PRODUÇÃO DE SENTIDOS NO CONTEXTO DA SURDOCEGUEIRA</t>
+          <t>A IMPORTÂNCIA DA LITERATURA SURDA PARA O ENSINO DE LIBRAS</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Ronna Freitas</t>
+          <t>Patricia Barreto Mainardi Maeso</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Terça</t>
+          <t>Segunda</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -3430,19 +3491,19 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Debora Santos Resende</t>
+          <t>Maria Jacinta Pfeiffer</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>AS PLATAFORMAS DE ENSINO DE INGLÊS DA REDE PÚBLICA PARANAENSE FRENTE AOS DOCUMENTOS OFICIAIS</t>
+          <t>O tempo como fator de conversão: Uma canção de natal de Charles Dickens</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Rosita Maria Bastos dos Santos</t>
+          <t>Pâmela Cristina Pereira Gonzaga</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -3467,24 +3528,24 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Orientador</t>
+          <t>Membro</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Martha Caixeta Cardoso</t>
+          <t>Amanda Rafaelly de Paula Rocha</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>A ESCRITA AUTORAL COMO ESTRATÉGIA PEDAGÓGICA NA LEITURA E PRODUÇÃO DE TEXTOS: UM RELATO DE EXPERIÊNCIA NO PROJETO DE EXTENSÃO</t>
+          <t>COMUNICAÇÃO SOCIAL HÁPTICA: LÍNGUA, INTERAÇÃO E PRODUÇÃO DE SENTIDOS NO CONTEXTO DA SURDOCEGUEIRA</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Rosita Maria Bastos dos Santos</t>
+          <t>Ronna Freitas</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -3499,34 +3560,34 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>16:10</t>
+          <t>13:50</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>B202</t>
+          <t>B201</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Orientador</t>
+          <t>Membro</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>João Pedro Mendes Santos</t>
+          <t>Debora Santos Resende</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>Entre a universidade e a sala de aula: memórias e reflexões sobre a construção docente</t>
+          <t>AS PLATAFORMAS DE ENSINO DE INGLÊS DA REDE PÚBLICA PARANAENSE FRENTE AOS DOCUMENTOS OFICIAIS</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Rúbia Carla da Silva</t>
+          <t>Rosita Maria Bastos dos Santos</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -3541,7 +3602,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>13:50</t>
+          <t>16:10</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -3556,24 +3617,24 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Amanda Rafaelly de Paula Rocha</t>
+          <t>João Pedro Mendes Santos</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>COMUNICAÇÃO SOCIAL HÁPTICA: LÍNGUA, INTERAÇÃO E PRODUÇÃO DE SENTIDOS NO CONTEXTO DA SURDOCEGUEIRA</t>
+          <t>Entre a universidade e a sala de aula: memórias e reflexões sobre a construção docente</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Rúbia Carla da Silva</t>
+          <t>Rosita Maria Bastos dos Santos</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Segunda</t>
+          <t>Terça</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -3588,7 +3649,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>B204</t>
+          <t>B203</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -3598,19 +3659,19 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Thyelle Francine Braz de Proença</t>
+          <t>Martha Caixeta Cardoso</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>A IMPORTÂNCIA DA LITERATURA SURDA PARA O ENSINO DE LIBRAS</t>
+          <t>A ESCRITA AUTORAL COMO ESTRATÉGIA PEDAGÓGICA NA LEITURA E PRODUÇÃO DE TEXTOS: UM RELATO DE EXPERIÊNCIA NO PROJETO DE EXTENSÃO</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Rúbia Carla da Silva e Djane Antonucci Correa</t>
+          <t>Rúbia Carla da Silva</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -3652,12 +3713,12 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Shirley Vilhalva</t>
+          <t>Rúbia Carla da Silva</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Segunda</t>
+          <t>Terça</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -3667,39 +3728,39 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>13:50</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>B203</t>
+          <t>B202</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Membro</t>
+          <t>Orientador</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Marcos Vinicius Matias</t>
+          <t>Thyelle Francine Braz de Proença</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>ENTRE MÃOS E TERRITÓRIOS: LÍNGUAS INDÍGENAS DE SINAIS E SINGULARIDADES/IDENTIDADES DE INDÍGENAS SURDOS</t>
+          <t>A IMPORTÂNCIA DA LITERATURA SURDA PARA O ENSINO DE LIBRAS</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Silvely Brandes</t>
+          <t>Rúbia Carla da Silva</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Segunda</t>
+          <t>Terça</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -3709,7 +3770,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>16:10</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -3719,29 +3780,29 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Membro</t>
+          <t>Orientador</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Isabela Delgobo Champoski</t>
+          <t>Amanda Rafaelly de Paula Rocha</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>A proibição do celular em sala de aula: análise da aplicação da Lei 15.100/2025 em escolas públicas (2024-2025)</t>
+          <t>COMUNICAÇÃO SOCIAL HÁPTICA: LÍNGUA, INTERAÇÃO E PRODUÇÃO DE SENTIDOS NO CONTEXTO DA SURDOCEGUEIRA</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Silvely Brandes</t>
+          <t>Shirley Vilhalva</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Terça</t>
+          <t>Segunda</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -3751,27 +3812,27 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>13:50</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>B202</t>
+          <t>B203</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Orientador</t>
+          <t>Membro</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>Debora Santos Resende</t>
+          <t>Marcos Vinicius Matias</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>AS PLATAFORMAS DE ENSINO DE INGLÊS DA REDE PÚBLICA PARANAENSE FRENTE AOS DOCUMENTOS OFICIAIS</t>
+          <t>ENTRE MÃOS E TERRITÓRIOS: LÍNGUAS INDÍGENAS DE SINAIS E SINGULARIDADES/IDENTIDADES DE INDÍGENAS SURDOS</t>
         </is>
       </c>
     </row>
@@ -3783,7 +3844,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Terça</t>
+          <t>Segunda</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -3798,34 +3859,34 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>B203</t>
+          <t>B202</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Orientador</t>
+          <t>Membro</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>PEDRO MEYER KOPP</t>
+          <t>Isabela Delgobo Champoski</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>A TRADUÇÃO AUTOMÁTICA DENTRO DE JOGOS ELETRÔNICOS NA PLATAFORMA ROBLOX: UMA ANÁLISE QUALITATIVA</t>
+          <t>A proibição do celular em sala de aula: análise da aplicação da Lei 15.100/2025 em escolas públicas (2024-2025)</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>TILSP - Cristiane Ribeiro Rocha</t>
+          <t>Silvely Brandes</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Segunda</t>
+          <t>Terça</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -3835,39 +3896,39 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>16:10</t>
+          <t>13:50</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>B204</t>
+          <t>B201</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Membro</t>
+          <t>Orientador</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>Thyelle Francine Braz de Proença</t>
+          <t>Debora Santos Resende</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>A IMPORTÂNCIA DA LITERATURA SURDA PARA O ENSINO DE LIBRAS</t>
+          <t>AS PLATAFORMAS DE ENSINO DE INGLÊS DA REDE PÚBLICA PARANAENSE FRENTE AOS DOCUMENTOS OFICIAIS</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>TILSP - Marcelo Oliveira Bleme</t>
+          <t>Silvely Brandes</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Segunda</t>
+          <t>Terça</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -3882,22 +3943,22 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>B203</t>
+          <t>B201</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Membro</t>
+          <t>Orientador</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>Marcos Vinicius Matias</t>
+          <t>PEDRO MEYER KOPP</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>ENTRE MÃOS E TERRITÓRIOS: LÍNGUAS INDÍGENAS DE SINAIS E SINGULARIDADES/IDENTIDADES DE INDÍGENAS SURDOS</t>
+          <t>A TRADUÇÃO AUTOMÁTICA DENTRO DE JOGOS ELETRÔNICOS NA PLATAFORMA ROBLOX: UMA ANÁLISE QUALITATIVA</t>
         </is>
       </c>
     </row>
@@ -3909,7 +3970,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Segunda</t>
+          <t>Terça</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -3919,12 +3980,12 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>16:10</t>
+          <t>13:50</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>B204</t>
+          <t>B202</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -3946,40 +4007,82 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
+          <t>Álvaro Kasuaki Fujihara</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Terça</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>VESPERTINO</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>B201</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>Membro</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>PEDRO MEYER KOPP</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>A TRADUÇÃO AUTOMÁTICA DENTRO DE JOGOS ELETRÔNICOS NA PLATAFORMA ROBLOX: UMA ANÁLISE QUALITATIVA</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
           <t>Ályda Henrietta Zomer</t>
         </is>
       </c>
-      <c r="B58" t="inlineStr">
+      <c r="B59" t="inlineStr">
         <is>
           <t>Segunda</t>
         </is>
       </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>VESPERTINO</t>
-        </is>
-      </c>
-      <c r="D58" t="inlineStr">
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>VESPERTINO</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
         <is>
           <t>16:10</t>
         </is>
       </c>
-      <c r="E58" t="inlineStr">
+      <c r="E59" t="inlineStr">
         <is>
           <t>B202</t>
         </is>
       </c>
-      <c r="F58" t="inlineStr">
+      <c r="F59" t="inlineStr">
         <is>
           <t>Membro</t>
         </is>
       </c>
-      <c r="G58" t="inlineStr">
+      <c r="G59" t="inlineStr">
         <is>
           <t>Isabela Delgobo Champoski</t>
         </is>
       </c>
-      <c r="H58" t="inlineStr">
+      <c r="H59" t="inlineStr">
         <is>
           <t>A proibição do celular em sala de aula: análise da aplicação da Lei 15.100/2025 em escolas públicas (2024-2025)</t>
         </is>
@@ -4044,7 +4147,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Segunda</t>
+          <t>Terça</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -4054,12 +4157,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>13:50</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>B204</t>
+          <t>B202</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -4118,7 +4221,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Segunda</t>
+          <t>Terça</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -4128,12 +4231,12 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>16:10</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>B204</t>
+          <t>B202</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -4170,7 +4273,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>B202</t>
+          <t>B201</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -4377,7 +4480,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Terça</t>
+          <t>Segunda</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -4392,7 +4495,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>B202</t>
+          <t>B204</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -4471,7 +4574,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Rúbia Carla da Silva e Djane Antonucci Correa</t>
+          <t>Rúbia Carla da Silva</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -4535,12 +4638,12 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>16:10</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>B202</t>
+          <t>B203</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -4609,12 +4712,12 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>16:10</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>B203</t>
+          <t>B201</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -4673,7 +4776,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Segunda</t>
+          <t>Terça</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -4683,12 +4786,12 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>16:10</t>
+          <t>13:50</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>B204</t>
+          <t>B202</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -4751,12 +4854,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>B202</t>
+          <t>B201</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Segunda</t>
+          <t>Terça</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -4771,24 +4874,24 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Maria Jacinta Pfeiffer</t>
+          <t>Debora Santos Resende</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Giuliano Lellis Ito Santos</t>
+          <t>Silvely Brandes</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>B202</t>
+          <t>B201</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Segunda</t>
+          <t>Terça</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -4803,12 +4906,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Rodrigo Paes</t>
+          <t>PEDRO MEYER KOPP</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Giuliano Lellis Ito Santos</t>
+          <t>Silvely Brandes</t>
         </is>
       </c>
     </row>
@@ -4830,12 +4933,12 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>16:10</t>
+          <t>13:50</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Isabela Delgobo Champoski</t>
+          <t>Maria Jacinta Pfeiffer</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -4852,7 +4955,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Terça</t>
+          <t>Segunda</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -4862,17 +4965,17 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>13:50</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Debora Santos Resende</t>
+          <t>Rodrigo Paes</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Silvely Brandes</t>
+          <t>Giuliano Lellis Ito Santos</t>
         </is>
       </c>
     </row>
@@ -4884,7 +4987,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Terça</t>
+          <t>Segunda</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -4894,17 +4997,17 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>16:10</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Martha Caixeta Cardoso</t>
+          <t>Isabela Delgobo Champoski</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Rosita Maria Bastos dos Santos</t>
+          <t>Giuliano Lellis Ito Santos</t>
         </is>
       </c>
     </row>
@@ -4926,29 +5029,29 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>16:10</t>
+          <t>13:50</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>João Pedro Mendes Santos</t>
+          <t>Thyelle Francine Braz de Proença</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Rosita Maria Bastos dos Santos</t>
+          <t>Rúbia Carla da Silva</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>B203</t>
+          <t>B202</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Segunda</t>
+          <t>Terça</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -4958,29 +5061,29 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>13:50</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Elise Thaynara-Yvian Mendes Christofoli</t>
+          <t>Amanda Rafaelly de Paula Rocha</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Letícia Fraga</t>
+          <t>Rúbia Carla da Silva</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>B203</t>
+          <t>B202</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Segunda</t>
+          <t>Terça</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -4990,17 +5093,17 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>16:10</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Marcos Vinicius Matias</t>
+          <t>CLAUDINEIA MACHADO DE OLIVEIRA</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Rúbia Carla da Silva e Djane Antonucci Correa</t>
+          <t>Andressa França</t>
         </is>
       </c>
     </row>
@@ -5022,12 +5125,12 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>16:10</t>
+          <t>13:50</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Henrique Leal Rodrigues</t>
+          <t>Elise Thaynara-Yvian Mendes Christofoli</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -5044,7 +5147,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Terça</t>
+          <t>Segunda</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -5054,17 +5157,17 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>13:50</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Naiara Karin de Ramos</t>
+          <t>Marcos Vinicius Matias</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Dilma Heloisa Santos</t>
+          <t>Rúbia Carla da Silva</t>
         </is>
       </c>
     </row>
@@ -5076,7 +5179,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Terça</t>
+          <t>Segunda</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -5086,17 +5189,17 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>16:10</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>GRACIELY CRISTINY MATOS VIEIRA</t>
+          <t>Henrique Leal Rodrigues</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Ligia Paula Couto</t>
+          <t>Letícia Fraga</t>
         </is>
       </c>
     </row>
@@ -5118,29 +5221,29 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>16:10</t>
+          <t>13:50</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>PEDRO MEYER KOPP</t>
+          <t>Naiara Karin de Ramos</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Silvely Brandes</t>
+          <t>Dilma Heloisa Santos</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>B204</t>
+          <t>B203</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Segunda</t>
+          <t>Terça</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -5150,29 +5253,29 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>13:50</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Amanda Rafaelly de Paula Rocha</t>
+          <t>GRACIELY CRISTINY MATOS VIEIRA</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Rúbia Carla da Silva</t>
+          <t>Ligia Paula Couto</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>B204</t>
+          <t>B203</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Segunda</t>
+          <t>Terça</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -5182,17 +5285,17 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>16:10</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>CLAUDINEIA MACHADO DE OLIVEIRA</t>
+          <t>Martha Caixeta Cardoso</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Andressa França</t>
+          <t>Rosita Maria Bastos dos Santos</t>
         </is>
       </c>
     </row>
@@ -5219,12 +5322,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Thyelle Francine Braz de Proença</t>
+          <t>João Pedro Mendes Santos</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Rúbia Carla da Silva</t>
+          <t>Rosita Maria Bastos dos Santos</t>
         </is>
       </c>
     </row>

</xml_diff>